<commit_message>
Added new RDF data schemes and visual schemes for education-table08-12, fixed XLSX spreadsheets for education-table08-12
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/education-table08.xlsx
+++ b/sources/table_normalization/xlsx/education-table08.xlsx
@@ -429,9 +429,6 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -479,55 +476,58 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal 3" xfId="1"/>
@@ -1104,7 +1104,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1113,69 +1113,69 @@
     </row>
     <row r="3" spans="1:15" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="48"/>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="32" t="s">
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="33"/>
-      <c r="O3" s="33"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
     </row>
     <row r="4" spans="1:15" s="1" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="41" t="s">
+      <c r="G4" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="42" t="s">
+      <c r="H4" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="41" t="s">
+      <c r="I4" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="41" t="s">
+      <c r="J4" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="K4" s="41" t="s">
+      <c r="K4" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="41" t="s">
+      <c r="L4" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="41" t="s">
+      <c r="M4" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="41" t="s">
+      <c r="N4" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="42" t="s">
+      <c r="O4" s="46" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       <c r="G5" s="9">
         <v>290660</v>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="21">
         <v>860200</v>
       </c>
       <c r="I5" s="9">
@@ -1222,7 +1222,7 @@
       <c r="N5" s="9">
         <v>117290</v>
       </c>
-      <c r="O5" s="22">
+      <c r="O5" s="21">
         <v>481800</v>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       <c r="G6" s="11">
         <v>282080</v>
       </c>
-      <c r="H6" s="23">
+      <c r="H6" s="22">
         <v>721700</v>
       </c>
       <c r="I6" s="11">
@@ -1269,7 +1269,7 @@
       <c r="N6" s="11">
         <v>110150</v>
       </c>
-      <c r="O6" s="23">
+      <c r="O6" s="22">
         <v>385200</v>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       <c r="G7" s="13">
         <v>11600</v>
       </c>
-      <c r="H7" s="24">
+      <c r="H7" s="23">
         <v>207400</v>
       </c>
       <c r="I7" s="13">
@@ -1316,94 +1316,94 @@
       <c r="N7" s="13">
         <v>4850</v>
       </c>
-      <c r="O7" s="24">
+      <c r="O7" s="23">
         <v>149400</v>
       </c>
     </row>
     <row r="8" spans="1:15" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="14">
         <v>684750</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="14">
         <v>36810</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="14">
         <v>26470</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="14">
         <v>180900</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="14">
         <v>880</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="14">
         <v>382280</v>
       </c>
-      <c r="H8" s="25">
+      <c r="H8" s="24">
         <v>1312100</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="14">
         <v>462770</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="14">
         <v>27950</v>
       </c>
-      <c r="K8" s="15">
+      <c r="K8" s="14">
         <v>18870</v>
       </c>
-      <c r="L8" s="15">
+      <c r="L8" s="14">
         <v>130620</v>
       </c>
-      <c r="M8" s="15">
+      <c r="M8" s="14">
         <v>700</v>
       </c>
-      <c r="N8" s="15">
+      <c r="N8" s="14">
         <v>171660</v>
       </c>
-      <c r="O8" s="25">
+      <c r="O8" s="24">
         <v>812600</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="43" t="s">
+      <c r="A9" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="44"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="44"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="44"/>
-      <c r="J9" s="44"/>
-      <c r="K9" s="44"/>
-      <c r="L9" s="44"/>
-      <c r="M9" s="44"/>
-      <c r="N9" s="44"/>
-      <c r="O9" s="45"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="34"/>
+      <c r="K9" s="34"/>
+      <c r="L9" s="34"/>
+      <c r="M9" s="34"/>
+      <c r="N9" s="34"/>
+      <c r="O9" s="35"/>
     </row>
     <row r="10" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="46" t="s">
+      <c r="A10" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
-      <c r="D10" s="46"/>
-      <c r="E10" s="46"/>
-      <c r="F10" s="46"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="46"/>
-      <c r="I10" s="46"/>
-      <c r="J10" s="46"/>
-      <c r="K10" s="46"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="46"/>
-      <c r="N10" s="46"/>
-      <c r="O10" s="46"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="45"/>
+      <c r="J10" s="45"/>
+      <c r="K10" s="45"/>
+      <c r="L10" s="45"/>
+      <c r="M10" s="45"/>
+      <c r="N10" s="45"/>
+      <c r="O10" s="45"/>
     </row>
     <row r="11" spans="1:15" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11"/>
@@ -1782,187 +1782,187 @@
     <row r="33" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" spans="1:16" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="35" spans="1:16" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="34"/>
-      <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="34"/>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="34"/>
-      <c r="H35" s="34"/>
-      <c r="I35" s="34"/>
-      <c r="J35" s="34"/>
-      <c r="K35" s="34"/>
-      <c r="L35" s="34"/>
-      <c r="M35" s="34"/>
-      <c r="N35" s="34"/>
-      <c r="O35" s="34"/>
+      <c r="A35" s="37"/>
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="37"/>
+      <c r="I35" s="37"/>
+      <c r="J35" s="37"/>
+      <c r="K35" s="37"/>
+      <c r="L35" s="37"/>
+      <c r="M35" s="37"/>
+      <c r="N35" s="37"/>
+      <c r="O35" s="37"/>
     </row>
     <row r="36" spans="1:16" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="17"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
-      <c r="G36" s="17"/>
-      <c r="H36" s="17"/>
-      <c r="I36" s="17"/>
-      <c r="J36" s="17"/>
-      <c r="K36" s="17"/>
-      <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-      <c r="N36" s="17"/>
-      <c r="O36" s="17"/>
+      <c r="A36" s="16"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="16"/>
+      <c r="K36" s="16"/>
+      <c r="L36" s="16"/>
+      <c r="M36" s="16"/>
+      <c r="N36" s="16"/>
+      <c r="O36" s="16"/>
     </row>
     <row r="37" spans="1:16" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="17"/>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="17"/>
-      <c r="G37" s="17"/>
-      <c r="H37" s="17"/>
-      <c r="I37" s="18"/>
-      <c r="J37" s="18"/>
-      <c r="K37" s="18"/>
-      <c r="L37" s="18"/>
-      <c r="M37" s="18"/>
-      <c r="N37" s="26"/>
-      <c r="O37" s="27"/>
+      <c r="A37" s="16"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+      <c r="I37" s="17"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="17"/>
+      <c r="M37" s="17"/>
+      <c r="N37" s="25"/>
+      <c r="O37" s="26"/>
     </row>
     <row r="38" spans="1:16" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="35"/>
-      <c r="B38" s="35"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="35"/>
-      <c r="F38" s="35"/>
-      <c r="G38" s="35"/>
-      <c r="H38" s="35"/>
-      <c r="I38" s="35"/>
-      <c r="J38" s="35"/>
-      <c r="K38" s="35"/>
-      <c r="L38" s="35"/>
-      <c r="M38" s="35"/>
-      <c r="N38" s="35"/>
-      <c r="O38" s="35"/>
+      <c r="A38" s="41"/>
+      <c r="B38" s="41"/>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="41"/>
+      <c r="F38" s="41"/>
+      <c r="G38" s="41"/>
+      <c r="H38" s="41"/>
+      <c r="I38" s="41"/>
+      <c r="J38" s="41"/>
+      <c r="K38" s="41"/>
+      <c r="L38" s="41"/>
+      <c r="M38" s="41"/>
+      <c r="N38" s="41"/>
+      <c r="O38" s="41"/>
     </row>
     <row r="39" spans="1:16" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="34"/>
-      <c r="B39" s="36"/>
-      <c r="C39" s="36"/>
-      <c r="D39" s="36"/>
-      <c r="E39" s="36"/>
-      <c r="F39" s="36"/>
-      <c r="G39" s="36"/>
-      <c r="H39" s="36"/>
-      <c r="I39" s="36"/>
-      <c r="J39" s="16"/>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="26"/>
-      <c r="N39" s="27"/>
-      <c r="O39" s="28"/>
+      <c r="A39" s="37"/>
+      <c r="B39" s="38"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="38"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="38"/>
+      <c r="J39" s="15"/>
+      <c r="K39" s="15"/>
+      <c r="L39" s="15"/>
+      <c r="M39" s="25"/>
+      <c r="N39" s="26"/>
+      <c r="O39" s="27"/>
     </row>
     <row r="40" spans="1:16" s="5" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="37"/>
-      <c r="B40" s="37"/>
-      <c r="C40" s="37"/>
-      <c r="D40" s="37"/>
-      <c r="E40" s="37"/>
-      <c r="F40" s="37"/>
-      <c r="G40" s="37"/>
-      <c r="H40" s="37"/>
-      <c r="I40" s="37"/>
-      <c r="J40" s="37"/>
-      <c r="K40" s="37"/>
-      <c r="L40" s="38"/>
-      <c r="M40" s="38"/>
-      <c r="N40" s="38"/>
-      <c r="O40" s="38"/>
+      <c r="A40" s="39"/>
+      <c r="B40" s="39"/>
+      <c r="C40" s="39"/>
+      <c r="D40" s="39"/>
+      <c r="E40" s="39"/>
+      <c r="F40" s="39"/>
+      <c r="G40" s="39"/>
+      <c r="H40" s="39"/>
+      <c r="I40" s="39"/>
+      <c r="J40" s="39"/>
+      <c r="K40" s="39"/>
+      <c r="L40" s="40"/>
+      <c r="M40" s="40"/>
+      <c r="N40" s="40"/>
+      <c r="O40" s="40"/>
     </row>
     <row r="41" spans="1:16" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="38"/>
-      <c r="B41" s="38"/>
-      <c r="C41" s="38"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="38"/>
-      <c r="F41" s="38"/>
-      <c r="G41" s="38"/>
-      <c r="H41" s="38"/>
-      <c r="I41" s="38"/>
-      <c r="J41" s="38"/>
-      <c r="K41" s="38"/>
-      <c r="L41" s="38"/>
-      <c r="M41" s="38"/>
-      <c r="N41" s="38"/>
-      <c r="O41" s="38"/>
+      <c r="A41" s="40"/>
+      <c r="B41" s="40"/>
+      <c r="C41" s="40"/>
+      <c r="D41" s="40"/>
+      <c r="E41" s="40"/>
+      <c r="F41" s="40"/>
+      <c r="G41" s="40"/>
+      <c r="H41" s="40"/>
+      <c r="I41" s="40"/>
+      <c r="J41" s="40"/>
+      <c r="K41" s="40"/>
+      <c r="L41" s="40"/>
+      <c r="M41" s="40"/>
+      <c r="N41" s="40"/>
+      <c r="O41" s="40"/>
     </row>
     <row r="42" spans="1:16" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="35"/>
-      <c r="B42" s="38"/>
-      <c r="C42" s="38"/>
-      <c r="D42" s="38"/>
-      <c r="E42" s="38"/>
-      <c r="F42" s="38"/>
-      <c r="G42" s="38"/>
-      <c r="H42" s="38"/>
-      <c r="I42" s="38"/>
-      <c r="J42" s="38"/>
-      <c r="K42" s="38"/>
-      <c r="L42" s="38"/>
-      <c r="M42" s="38"/>
-      <c r="N42" s="38"/>
-      <c r="O42" s="38"/>
-      <c r="P42" s="29"/>
+      <c r="A42" s="41"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="40"/>
+      <c r="E42" s="40"/>
+      <c r="F42" s="40"/>
+      <c r="G42" s="40"/>
+      <c r="H42" s="40"/>
+      <c r="I42" s="40"/>
+      <c r="J42" s="40"/>
+      <c r="K42" s="40"/>
+      <c r="L42" s="40"/>
+      <c r="M42" s="40"/>
+      <c r="N42" s="40"/>
+      <c r="O42" s="40"/>
+      <c r="P42" s="28"/>
     </row>
     <row r="43" spans="1:16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="19"/>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
-      <c r="E43" s="20"/>
-      <c r="F43" s="20"/>
-      <c r="G43" s="20"/>
-      <c r="H43" s="20"/>
-      <c r="I43" s="20"/>
-      <c r="J43" s="20"/>
-      <c r="K43" s="20"/>
-      <c r="L43" s="20"/>
-      <c r="M43" s="20"/>
-      <c r="N43" s="20"/>
-      <c r="O43" s="20"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="19"/>
+      <c r="C43" s="19"/>
+      <c r="D43" s="19"/>
+      <c r="E43" s="19"/>
+      <c r="F43" s="19"/>
+      <c r="G43" s="19"/>
+      <c r="H43" s="19"/>
+      <c r="I43" s="19"/>
+      <c r="J43" s="19"/>
+      <c r="K43" s="19"/>
+      <c r="L43" s="19"/>
+      <c r="M43" s="19"/>
+      <c r="N43" s="19"/>
+      <c r="O43" s="19"/>
     </row>
     <row r="44" spans="1:16" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="39"/>
-      <c r="B44" s="39"/>
-      <c r="C44" s="39"/>
-      <c r="D44" s="39"/>
-      <c r="E44" s="39"/>
-      <c r="F44" s="39"/>
-      <c r="G44" s="39"/>
-      <c r="H44" s="39"/>
-      <c r="I44" s="39"/>
-      <c r="J44" s="21"/>
-      <c r="K44" s="21"/>
-      <c r="L44" s="21"/>
-      <c r="M44" s="30"/>
-      <c r="N44" s="31"/>
+      <c r="A44" s="42"/>
+      <c r="B44" s="42"/>
+      <c r="C44" s="42"/>
+      <c r="D44" s="42"/>
+      <c r="E44" s="42"/>
+      <c r="F44" s="42"/>
+      <c r="G44" s="42"/>
+      <c r="H44" s="42"/>
+      <c r="I44" s="42"/>
+      <c r="J44" s="20"/>
+      <c r="K44" s="20"/>
+      <c r="L44" s="20"/>
+      <c r="M44" s="29"/>
+      <c r="N44" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="I3:O3"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A35:O35"/>
+    <mergeCell ref="A38:O38"/>
     <mergeCell ref="A39:I39"/>
     <mergeCell ref="A40:O40"/>
     <mergeCell ref="A41:O41"/>
     <mergeCell ref="A42:O42"/>
     <mergeCell ref="A44:I44"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="I3:O3"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A35:O35"/>
-    <mergeCell ref="A38:O38"/>
   </mergeCells>
   <pageMargins left="0.39370078740157499" right="0.47244094488188998" top="0.98425196850393704" bottom="0.98425196850393704" header="0.47244094488188998" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="58" orientation="landscape"/>

</xml_diff>